<commit_message>
Finished an iteration on report processing.
</commit_message>
<xml_diff>
--- a/PythonScripts/Caffé_Dal_1927_Kereskedelemi_és_Szolgáltató_Korlátolt_Felelősségű_Társaság_Beszamolo_Elemzes.xlsx
+++ b/PythonScripts/Caffé_Dal_1927_Kereskedelemi_és_Szolgáltató_Korlátolt_Felelősségű_Társaság_Beszamolo_Elemzes.xlsx
@@ -1348,34 +1348,34 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>62</v>
+        <v>182</v>
       </c>
       <c r="C26" t="n">
-        <v>63</v>
+        <v>183</v>
       </c>
       <c r="D26" t="n">
-        <v>64</v>
+        <v>184</v>
       </c>
       <c r="E26" t="n">
-        <v>65</v>
+        <v>185</v>
       </c>
       <c r="F26" t="n">
-        <v>66</v>
+        <v>186</v>
       </c>
       <c r="G26" t="n">
-        <v>67</v>
+        <v>187</v>
       </c>
       <c r="H26" t="n">
-        <v>68</v>
+        <v>188</v>
       </c>
       <c r="I26" t="n">
-        <v>69</v>
+        <v>189</v>
       </c>
       <c r="J26" t="n">
-        <v>70</v>
+        <v>190</v>
       </c>
       <c r="K26" t="n">
-        <v>71</v>
+        <v>191</v>
       </c>
     </row>
     <row r="27">
@@ -7304,7 +7304,9 @@
           <t>MUTATO: Vagyon változása (%)</t>
         </is>
       </c>
-      <c r="B187" t="inlineStr"/>
+      <c r="B187" t="n">
+        <v>0</v>
+      </c>
       <c r="C187" t="n">
         <v>26.02338519992762</v>
       </c>

</xml_diff>